<commit_message>
implemented hierarchy in extent reports
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata.xlsx
+++ b/src/test/resources/testdata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maiya\IdeaProjects\KDE\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maiya\IdeaProjects\keyword_driven_framework_TestNG\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{191099FB-1E18-48C6-AB1A-23D2C005334F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECAE57CD-6754-4838-849D-E3E44FBE246A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8751E216-6B08-4D68-A5A1-62EEF9F6395D}"/>
   </bookViews>

</xml_diff>